<commit_message>
Protège le classeur Excel et améliore la saisie multi-lignes
- Feuille protégée (mot de passe PEI) : seuls les champs à compléter et les
  cases à cocher sont modifiables ; libellés, cellules pré-remplies et totaux
  sont verrouillés contre toute modification accidentelle
- Sélection limitée aux cellules déverrouillées : Entrée/Tab passe d'un champ
  à remplir au suivant
- Retour à la ligne automatique activé et zones de saisie agrandies (pour
  plusieurs lignes : Alt+Entrée)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FVySUXCR7Npo3V7p3PjL1D
</commit_message>
<xml_diff>
--- a/PEI_a_completer.xlsx
+++ b/PEI_a_completer.xlsx
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -135,13 +135,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -160,8 +165,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -579,10 +585,10 @@
         </is>
       </c>
       <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -591,10 +597,10 @@
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -603,10 +609,10 @@
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -615,10 +621,10 @@
         </is>
       </c>
       <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -627,20 +633,20 @@
         </is>
       </c>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Raisons du placement</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="8" t="n"/>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -661,64 +667,64 @@
           <t>Type de mandat (cocher)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>SAJ</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>SPJ</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>Tribunal</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Lieu (SPJ / SAJ / Tribunal)</t>
         </is>
       </c>
       <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Directrice / conseillère</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Déléguée</t>
         </is>
       </c>
       <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
+      <c r="G16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -726,32 +732,32 @@
           <t>Prise en charge (cocher)</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>F.A.</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>Frais</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>SAAF</t>
         </is>
@@ -763,46 +769,46 @@
           <t>Allocation forfaitaire allouée à (cocher)</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>Maman</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Papa</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>Enfant</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Décisions de la dernière formalisation</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="8" t="n"/>
+    <row r="20" ht="46" customHeight="1">
+      <c r="A20" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -818,129 +824,129 @@
       <c r="G23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Besoin</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Objectifs de travail (court / moyen / long terme)</t>
         </is>
       </c>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="n"/>
-    </row>
-    <row r="25" ht="38" customHeight="1">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="13" t="n"/>
+    </row>
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Besoins physiologiques – sommeil – alimentation – santé (suivi médical, vaccins, dentiste…)</t>
         </is>
       </c>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-    </row>
-    <row r="26" ht="38" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="46" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Sécurité – protection – stabilité (repères, limites)</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-    </row>
-    <row r="27" ht="38" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="46" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Affectif – relation d'attachement – appartenance</t>
         </is>
       </c>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="8" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-    </row>
-    <row r="28" ht="38" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="9" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="46" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>Estime de soi – épanouissement</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="8" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
-    </row>
-    <row r="29" ht="38" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="9" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="9" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+    </row>
+    <row r="29" ht="46" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Apprentissage – formation</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="8" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="n"/>
-    </row>
-    <row r="30" ht="38" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+    </row>
+    <row r="30" ht="46" customHeight="1">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>Développement des compétences</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-    </row>
-    <row r="31" ht="38" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="n"/>
+    </row>
+    <row r="31" ht="46" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Appartenance à un réseau social</t>
         </is>
       </c>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="8" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="n"/>
-    </row>
-    <row r="32" ht="38" customHeight="1">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+    </row>
+    <row r="32" ht="46" customHeight="1">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Développer son autonomie – sa responsabilité</t>
         </is>
       </c>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="8" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -956,168 +962,168 @@
       <c r="G35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>Élément</t>
         </is>
       </c>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="12" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>Objectifs de travail (court / moyen / long terme)</t>
         </is>
       </c>
-      <c r="F36" s="12" t="n"/>
-      <c r="G36" s="12" t="n"/>
-    </row>
-    <row r="37" ht="38" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="13" t="n"/>
+    </row>
+    <row r="37" ht="46" customHeight="1">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>Situation actuelle</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="8" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="6" t="n"/>
-    </row>
-    <row r="38" ht="38" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="n"/>
+    </row>
+    <row r="38" ht="46" customHeight="1">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Disponibilité</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="8" t="n"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="8" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
-    </row>
-    <row r="39" ht="38" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="9" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="9" t="n"/>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="n"/>
+    </row>
+    <row r="39" ht="46" customHeight="1">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Collaboration</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="8" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="6" t="n"/>
-    </row>
-    <row r="40" ht="38" customHeight="1">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="n"/>
+    </row>
+    <row r="40" ht="46" customHeight="1">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t>Ouverture à la F.O.</t>
         </is>
       </c>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="8" t="n"/>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="8" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="6" t="n"/>
-    </row>
-    <row r="41" ht="38" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="B40" s="7" t="n"/>
+      <c r="C40" s="9" t="n"/>
+      <c r="D40" s="7" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="7" t="n"/>
+    </row>
+    <row r="41" ht="46" customHeight="1">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>À l'extérieur</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="8" t="n"/>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="8" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="6" t="n"/>
-    </row>
-    <row r="42" ht="38" customHeight="1">
-      <c r="A42" s="14" t="inlineStr">
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="9" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="7" t="n"/>
+    </row>
+    <row r="42" ht="46" customHeight="1">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>Éducation (souple, rigide…)</t>
         </is>
       </c>
-      <c r="B42" s="6" t="n"/>
-      <c r="C42" s="8" t="n"/>
-      <c r="D42" s="6" t="n"/>
-      <c r="E42" s="8" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="6" t="n"/>
-    </row>
-    <row r="43" ht="38" customHeight="1">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="B42" s="7" t="n"/>
+      <c r="C42" s="9" t="n"/>
+      <c r="D42" s="7" t="n"/>
+      <c r="E42" s="9" t="n"/>
+      <c r="F42" s="7" t="n"/>
+      <c r="G42" s="7" t="n"/>
+    </row>
+    <row r="43" ht="46" customHeight="1">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>Remise en question</t>
         </is>
       </c>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="8" t="n"/>
-      <c r="D43" s="6" t="n"/>
-      <c r="E43" s="8" t="n"/>
-      <c r="F43" s="6" t="n"/>
-      <c r="G43" s="6" t="n"/>
-    </row>
-    <row r="44" ht="38" customHeight="1">
-      <c r="A44" s="14" t="inlineStr">
+      <c r="B43" s="7" t="n"/>
+      <c r="C43" s="9" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="9" t="n"/>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="n"/>
+    </row>
+    <row r="44" ht="46" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>Relations famille élargie (fratrie, grands-parents…)</t>
         </is>
       </c>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="8" t="n"/>
-      <c r="D44" s="6" t="n"/>
-      <c r="E44" s="8" t="n"/>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="6" t="n"/>
-    </row>
-    <row r="45" ht="38" customHeight="1">
-      <c r="A45" s="14" t="inlineStr">
+      <c r="B44" s="7" t="n"/>
+      <c r="C44" s="9" t="n"/>
+      <c r="D44" s="7" t="n"/>
+      <c r="E44" s="9" t="n"/>
+      <c r="F44" s="7" t="n"/>
+      <c r="G44" s="7" t="n"/>
+    </row>
+    <row r="45" ht="46" customHeight="1">
+      <c r="A45" s="15" t="inlineStr">
         <is>
           <t>Réseau</t>
         </is>
       </c>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="8" t="n"/>
-      <c r="D45" s="6" t="n"/>
-      <c r="E45" s="8" t="n"/>
-      <c r="F45" s="6" t="n"/>
-      <c r="G45" s="6" t="n"/>
-    </row>
-    <row r="46" ht="38" customHeight="1">
-      <c r="A46" s="14" t="inlineStr">
+      <c r="B45" s="7" t="n"/>
+      <c r="C45" s="9" t="n"/>
+      <c r="D45" s="7" t="n"/>
+      <c r="E45" s="9" t="n"/>
+      <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="n"/>
+    </row>
+    <row r="46" ht="46" customHeight="1">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Couple</t>
         </is>
       </c>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="8" t="n"/>
-      <c r="D46" s="6" t="n"/>
-      <c r="E46" s="8" t="n"/>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="6" t="n"/>
-    </row>
-    <row r="47" ht="38" customHeight="1">
-      <c r="A47" s="14" t="inlineStr">
+      <c r="B46" s="7" t="n"/>
+      <c r="C46" s="9" t="n"/>
+      <c r="D46" s="7" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="7" t="n"/>
+      <c r="G46" s="7" t="n"/>
+    </row>
+    <row r="47" ht="46" customHeight="1">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>Rôles parentaux</t>
         </is>
       </c>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="8" t="n"/>
-      <c r="D47" s="6" t="n"/>
-      <c r="E47" s="8" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="6" t="n"/>
+      <c r="B47" s="7" t="n"/>
+      <c r="C47" s="9" t="n"/>
+      <c r="D47" s="7" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -1133,103 +1139,103 @@
       <c r="G50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>Élément</t>
         </is>
       </c>
-      <c r="B51" s="12" t="n"/>
-      <c r="C51" s="11" t="inlineStr">
+      <c r="B51" s="13" t="n"/>
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="D51" s="12" t="n"/>
-      <c r="E51" s="13" t="inlineStr">
+      <c r="D51" s="13" t="n"/>
+      <c r="E51" s="14" t="inlineStr">
         <is>
           <t>Objectifs de travail (court / moyen / long terme)</t>
         </is>
       </c>
-      <c r="F51" s="12" t="n"/>
-      <c r="G51" s="12" t="n"/>
-    </row>
-    <row r="52" ht="38" customHeight="1">
-      <c r="A52" s="14" t="inlineStr">
+      <c r="F51" s="13" t="n"/>
+      <c r="G51" s="13" t="n"/>
+    </row>
+    <row r="52" ht="46" customHeight="1">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>Situation actuelle</t>
         </is>
       </c>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="8" t="n"/>
-      <c r="D52" s="6" t="n"/>
-      <c r="E52" s="8" t="n"/>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="6" t="n"/>
-    </row>
-    <row r="53" ht="38" customHeight="1">
-      <c r="A53" s="14" t="inlineStr">
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="9" t="n"/>
+      <c r="D52" s="7" t="n"/>
+      <c r="E52" s="9" t="n"/>
+      <c r="F52" s="7" t="n"/>
+      <c r="G52" s="7" t="n"/>
+    </row>
+    <row r="53" ht="46" customHeight="1">
+      <c r="A53" s="15" t="inlineStr">
         <is>
           <t>Perception des parents</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="8" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="8" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="6" t="n"/>
-    </row>
-    <row r="54" ht="38" customHeight="1">
-      <c r="A54" s="14" t="inlineStr">
+      <c r="B53" s="7" t="n"/>
+      <c r="C53" s="9" t="n"/>
+      <c r="D53" s="7" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="F53" s="7" t="n"/>
+      <c r="G53" s="7" t="n"/>
+    </row>
+    <row r="54" ht="46" customHeight="1">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>Collaboration</t>
         </is>
       </c>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="8" t="n"/>
-      <c r="D54" s="6" t="n"/>
-      <c r="E54" s="8" t="n"/>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="6" t="n"/>
-    </row>
-    <row r="55" ht="38" customHeight="1">
-      <c r="A55" s="14" t="inlineStr">
+      <c r="B54" s="7" t="n"/>
+      <c r="C54" s="9" t="n"/>
+      <c r="D54" s="7" t="n"/>
+      <c r="E54" s="9" t="n"/>
+      <c r="F54" s="7" t="n"/>
+      <c r="G54" s="7" t="n"/>
+    </row>
+    <row r="55" ht="46" customHeight="1">
+      <c r="A55" s="15" t="inlineStr">
         <is>
           <t>Remise en question</t>
         </is>
       </c>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="8" t="n"/>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="8" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="6" t="n"/>
-    </row>
-    <row r="56" ht="38" customHeight="1">
-      <c r="A56" s="14" t="inlineStr">
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="9" t="n"/>
+      <c r="D55" s="7" t="n"/>
+      <c r="E55" s="9" t="n"/>
+      <c r="F55" s="7" t="n"/>
+      <c r="G55" s="7" t="n"/>
+    </row>
+    <row r="56" ht="46" customHeight="1">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t>D.R.P.</t>
         </is>
       </c>
-      <c r="B56" s="6" t="n"/>
-      <c r="C56" s="8" t="n"/>
-      <c r="D56" s="6" t="n"/>
-      <c r="E56" s="8" t="n"/>
-      <c r="F56" s="6" t="n"/>
-      <c r="G56" s="6" t="n"/>
-    </row>
-    <row r="57" ht="38" customHeight="1">
-      <c r="A57" s="14" t="inlineStr">
+      <c r="B56" s="7" t="n"/>
+      <c r="C56" s="9" t="n"/>
+      <c r="D56" s="7" t="n"/>
+      <c r="E56" s="9" t="n"/>
+      <c r="F56" s="7" t="n"/>
+      <c r="G56" s="7" t="n"/>
+    </row>
+    <row r="57" ht="46" customHeight="1">
+      <c r="A57" s="15" t="inlineStr">
         <is>
           <t>Autre</t>
         </is>
       </c>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="8" t="n"/>
-      <c r="D57" s="6" t="n"/>
-      <c r="E57" s="8" t="n"/>
-      <c r="F57" s="6" t="n"/>
-      <c r="G57" s="6" t="n"/>
+      <c r="B57" s="7" t="n"/>
+      <c r="C57" s="9" t="n"/>
+      <c r="D57" s="7" t="n"/>
+      <c r="E57" s="9" t="n"/>
+      <c r="F57" s="7" t="n"/>
+      <c r="G57" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -1245,30 +1251,30 @@
       <c r="G60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="inlineStr">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B61" s="12" t="n"/>
-      <c r="C61" s="12" t="n"/>
-      <c r="D61" s="12" t="n"/>
-      <c r="E61" s="13" t="inlineStr">
+      <c r="B61" s="13" t="n"/>
+      <c r="C61" s="13" t="n"/>
+      <c r="D61" s="13" t="n"/>
+      <c r="E61" s="14" t="inlineStr">
         <is>
           <t>Objectifs de travail (court / moyen / long terme)</t>
         </is>
       </c>
-      <c r="F61" s="12" t="n"/>
-      <c r="G61" s="12" t="n"/>
-    </row>
-    <row r="62" ht="50" customHeight="1">
-      <c r="A62" s="8" t="n"/>
-      <c r="B62" s="6" t="n"/>
-      <c r="C62" s="6" t="n"/>
-      <c r="D62" s="6" t="n"/>
-      <c r="E62" s="8" t="n"/>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="6" t="n"/>
+      <c r="F61" s="13" t="n"/>
+      <c r="G61" s="13" t="n"/>
+    </row>
+    <row r="62" ht="56" customHeight="1">
+      <c r="A62" s="9" t="n"/>
+      <c r="B62" s="7" t="n"/>
+      <c r="C62" s="7" t="n"/>
+      <c r="D62" s="7" t="n"/>
+      <c r="E62" s="9" t="n"/>
+      <c r="F62" s="7" t="n"/>
+      <c r="G62" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -1283,65 +1289,65 @@
       <c r="F65" s="4" t="n"/>
       <c r="G65" s="4" t="n"/>
     </row>
-    <row r="66" ht="32" customHeight="1">
+    <row r="66" ht="38" customHeight="1">
       <c r="A66" s="5" t="inlineStr">
         <is>
           <t>Enfant</t>
         </is>
       </c>
-      <c r="C66" s="8" t="n"/>
-      <c r="D66" s="6" t="n"/>
-      <c r="E66" s="6" t="n"/>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="6" t="n"/>
-    </row>
-    <row r="67" ht="32" customHeight="1">
+      <c r="C66" s="9" t="n"/>
+      <c r="D66" s="7" t="n"/>
+      <c r="E66" s="7" t="n"/>
+      <c r="F66" s="7" t="n"/>
+      <c r="G66" s="7" t="n"/>
+    </row>
+    <row r="67" ht="38" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
           <t>Famille d'accueil</t>
         </is>
       </c>
-      <c r="C67" s="8" t="n"/>
-      <c r="D67" s="6" t="n"/>
-      <c r="E67" s="6" t="n"/>
-      <c r="F67" s="6" t="n"/>
-      <c r="G67" s="6" t="n"/>
-    </row>
-    <row r="68" ht="32" customHeight="1">
+      <c r="C67" s="9" t="n"/>
+      <c r="D67" s="7" t="n"/>
+      <c r="E67" s="7" t="n"/>
+      <c r="F67" s="7" t="n"/>
+      <c r="G67" s="7" t="n"/>
+    </row>
+    <row r="68" ht="38" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
           <t>Famille d'origine</t>
         </is>
       </c>
-      <c r="C68" s="8" t="n"/>
-      <c r="D68" s="6" t="n"/>
-      <c r="E68" s="6" t="n"/>
-      <c r="F68" s="6" t="n"/>
-      <c r="G68" s="6" t="n"/>
-    </row>
-    <row r="69" ht="32" customHeight="1">
+      <c r="C68" s="9" t="n"/>
+      <c r="D68" s="7" t="n"/>
+      <c r="E68" s="7" t="n"/>
+      <c r="F68" s="7" t="n"/>
+      <c r="G68" s="7" t="n"/>
+    </row>
+    <row r="69" ht="38" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
           <t>D.R.P.</t>
         </is>
       </c>
-      <c r="C69" s="8" t="n"/>
-      <c r="D69" s="6" t="n"/>
-      <c r="E69" s="6" t="n"/>
-      <c r="F69" s="6" t="n"/>
-      <c r="G69" s="6" t="n"/>
-    </row>
-    <row r="70" ht="32" customHeight="1">
+      <c r="C69" s="9" t="n"/>
+      <c r="D69" s="7" t="n"/>
+      <c r="E69" s="7" t="n"/>
+      <c r="F69" s="7" t="n"/>
+      <c r="G69" s="7" t="n"/>
+    </row>
+    <row r="70" ht="38" customHeight="1">
       <c r="A70" s="5" t="inlineStr">
         <is>
           <t>Mandat</t>
         </is>
       </c>
-      <c r="C70" s="8" t="n"/>
-      <c r="D70" s="6" t="n"/>
-      <c r="E70" s="6" t="n"/>
-      <c r="F70" s="6" t="n"/>
-      <c r="G70" s="6" t="n"/>
+      <c r="C70" s="9" t="n"/>
+      <c r="D70" s="7" t="n"/>
+      <c r="E70" s="7" t="n"/>
+      <c r="F70" s="7" t="n"/>
+      <c r="G70" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -1357,39 +1363,39 @@
       <c r="G73" s="4" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="15" t="inlineStr">
+      <c r="A74" s="16" t="inlineStr">
         <is>
           <t>Enfants</t>
         </is>
       </c>
-      <c r="B74" s="15" t="inlineStr">
+      <c r="B74" s="16" t="inlineStr">
         <is>
           <t>Pts</t>
         </is>
       </c>
-      <c r="C74" s="15" t="inlineStr">
+      <c r="C74" s="16" t="inlineStr">
         <is>
           <t>F.A.</t>
         </is>
       </c>
-      <c r="D74" s="15" t="inlineStr">
+      <c r="D74" s="16" t="inlineStr">
         <is>
           <t>Pts</t>
         </is>
       </c>
-      <c r="E74" s="15" t="inlineStr">
+      <c r="E74" s="16" t="inlineStr">
         <is>
           <t>F.O.</t>
         </is>
       </c>
-      <c r="F74" s="15" t="inlineStr">
+      <c r="F74" s="16" t="inlineStr">
         <is>
           <t>Pts</t>
         </is>
       </c>
     </row>
     <row r="75" ht="78" customHeight="1">
-      <c r="A75" s="16" t="inlineStr">
+      <c r="A75" s="17" t="inlineStr">
         <is>
           <t>D.R.P.
   • Nombre
@@ -1399,22 +1405,22 @@
   • Type</t>
         </is>
       </c>
-      <c r="B75" s="17" t="n"/>
-      <c r="C75" s="16" t="inlineStr">
+      <c r="B75" s="18" t="n"/>
+      <c r="C75" s="17" t="inlineStr">
         <is>
           <t>D.R.P.</t>
         </is>
       </c>
-      <c r="D75" s="17" t="n"/>
-      <c r="E75" s="16" t="inlineStr">
+      <c r="D75" s="18" t="n"/>
+      <c r="E75" s="17" t="inlineStr">
         <is>
           <t>D.R.P.</t>
         </is>
       </c>
-      <c r="F75" s="17" t="n"/>
+      <c r="F75" s="18" t="n"/>
     </row>
     <row r="76" ht="70" customHeight="1">
-      <c r="A76" s="16" t="inlineStr">
+      <c r="A76" s="17" t="inlineStr">
         <is>
           <t>État de l'enfant :
   • Scolaire
@@ -1423,109 +1429,109 @@
   • Développement</t>
         </is>
       </c>
-      <c r="B76" s="17" t="n"/>
-      <c r="C76" s="16" t="inlineStr">
+      <c r="B76" s="18" t="n"/>
+      <c r="C76" s="17" t="inlineStr">
         <is>
           <t>Administratif
 Financier</t>
         </is>
       </c>
-      <c r="D76" s="17" t="n"/>
-      <c r="E76" s="16" t="inlineStr">
+      <c r="D76" s="18" t="n"/>
+      <c r="E76" s="17" t="inlineStr">
         <is>
           <t>Retour des parents</t>
         </is>
       </c>
-      <c r="F76" s="17" t="n"/>
+      <c r="F76" s="18" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="16" t="inlineStr">
+      <c r="A77" s="17" t="inlineStr">
         <is>
           <t>Bilan 6 mois</t>
         </is>
       </c>
-      <c r="B77" s="17" t="n"/>
-      <c r="C77" s="16" t="inlineStr">
+      <c r="B77" s="18" t="n"/>
+      <c r="C77" s="17" t="inlineStr">
         <is>
           <t>Bilan 6 mois</t>
         </is>
       </c>
-      <c r="D77" s="17" t="n"/>
-      <c r="E77" s="16" t="inlineStr">
+      <c r="D77" s="18" t="n"/>
+      <c r="E77" s="17" t="inlineStr">
         <is>
           <t>Bilan 6 mois</t>
         </is>
       </c>
-      <c r="F77" s="17" t="n"/>
+      <c r="F77" s="18" t="n"/>
     </row>
     <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="16" t="inlineStr">
+      <c r="A78" s="17" t="inlineStr">
         <is>
           <t>Réintégration</t>
         </is>
       </c>
-      <c r="B78" s="17" t="n"/>
-      <c r="C78" s="16" t="inlineStr">
+      <c r="B78" s="18" t="n"/>
+      <c r="C78" s="17" t="inlineStr">
         <is>
           <t>Réintégration</t>
         </is>
       </c>
-      <c r="D78" s="17" t="n"/>
-      <c r="E78" s="16" t="inlineStr">
+      <c r="D78" s="18" t="n"/>
+      <c r="E78" s="17" t="inlineStr">
         <is>
           <t>Réintégration</t>
         </is>
       </c>
-      <c r="F78" s="17" t="n"/>
+      <c r="F78" s="18" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="16" t="inlineStr">
+      <c r="A79" s="17" t="inlineStr">
         <is>
           <t>Préparation à la majorité</t>
         </is>
       </c>
-      <c r="B79" s="17" t="n"/>
-      <c r="C79" s="16" t="inlineStr">
+      <c r="B79" s="18" t="n"/>
+      <c r="C79" s="17" t="inlineStr">
         <is>
           <t>Préparation à la majorité</t>
         </is>
       </c>
-      <c r="D79" s="17" t="n"/>
-      <c r="E79" s="16" t="inlineStr">
+      <c r="D79" s="18" t="n"/>
+      <c r="E79" s="17" t="inlineStr">
         <is>
           <t>Préparation à la majorité</t>
         </is>
       </c>
-      <c r="F79" s="17" t="n"/>
+      <c r="F79" s="18" t="n"/>
     </row>
     <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="16" t="inlineStr">
+      <c r="A80" s="17" t="inlineStr">
         <is>
           <t>Travail de l'histoire</t>
         </is>
       </c>
-      <c r="B80" s="17" t="n"/>
-      <c r="C80" s="16" t="inlineStr">
+      <c r="B80" s="18" t="n"/>
+      <c r="C80" s="17" t="inlineStr">
         <is>
           <t>Recherche activités</t>
         </is>
       </c>
-      <c r="D80" s="17" t="n"/>
-      <c r="E80" s="16" t="inlineStr">
+      <c r="D80" s="18" t="n"/>
+      <c r="E80" s="17" t="inlineStr">
         <is>
           <t>Écrits autorité</t>
         </is>
       </c>
-      <c r="F80" s="17" t="n"/>
+      <c r="F80" s="18" t="n"/>
     </row>
     <row r="81" ht="60" customHeight="1">
-      <c r="A81" s="16" t="inlineStr">
+      <c r="A81" s="17" t="inlineStr">
         <is>
           <t>Autorité (écrits)</t>
         </is>
       </c>
-      <c r="B81" s="17" t="n"/>
-      <c r="C81" s="16" t="inlineStr">
+      <c r="B81" s="18" t="n"/>
+      <c r="C81" s="17" t="inlineStr">
         <is>
           <t>Besoin de sécurité
   • Accompagnement
@@ -1533,44 +1539,45 @@
   • Autorité</t>
         </is>
       </c>
-      <c r="D81" s="17" t="n"/>
-      <c r="E81" s="16" t="inlineStr"/>
-      <c r="F81" s="17" t="n"/>
+      <c r="D81" s="18" t="n"/>
+      <c r="E81" s="17" t="inlineStr"/>
+      <c r="F81" s="18" t="n"/>
     </row>
     <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="16" t="inlineStr">
+      <c r="A82" s="17" t="inlineStr">
         <is>
           <t>Déplacements</t>
         </is>
       </c>
-      <c r="B82" s="17" t="n"/>
-      <c r="C82" s="16" t="inlineStr"/>
-      <c r="D82" s="17" t="n"/>
-      <c r="E82" s="16" t="inlineStr"/>
-      <c r="F82" s="17" t="n"/>
+      <c r="B82" s="18" t="n"/>
+      <c r="C82" s="17" t="inlineStr"/>
+      <c r="D82" s="18" t="n"/>
+      <c r="E82" s="17" t="inlineStr"/>
+      <c r="F82" s="18" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="18" t="inlineStr">
+      <c r="A83" s="19" t="inlineStr">
         <is>
           <t>TOTAUX</t>
         </is>
       </c>
-      <c r="B83" s="19">
+      <c r="B83" s="20">
         <f>SUM(B75:B82)</f>
         <v/>
       </c>
-      <c r="C83" s="20" t="n"/>
-      <c r="D83" s="19">
+      <c r="C83" s="21" t="n"/>
+      <c r="D83" s="20">
         <f>SUM(D75:D82)</f>
         <v/>
       </c>
-      <c r="E83" s="20" t="n"/>
-      <c r="F83" s="19">
+      <c r="E83" s="21" t="n"/>
+      <c r="F83" s="20">
         <f>SUM(F75:F82)</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CDB4"/>
   <mergeCells count="85">
     <mergeCell ref="C68:G68"/>
     <mergeCell ref="F16:G16"/>

</xml_diff>

<commit_message>
Excel : rend les champs faciles à remplir (correctif protection)
- Autorise la sélection de toutes les cellules (selectLockedCells désactivé) :
  on peut cliquer partout ; seules les zones de saisie et les cases restent
  modifiables, le reste est en lecture seule
- Ajoute un léger fond bleuté sur toutes les zones à remplir pour les repérer
  facilement (sans cadre)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FVySUXCR7Npo3V7p3PjL1D
</commit_message>
<xml_diff>
--- a/PEI_a_completer.xlsx
+++ b/PEI_a_completer.xlsx
@@ -68,12 +68,17 @@
       <color rgb="002C5F7C"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1F6"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -96,7 +101,7 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00C9D3DA"/>
+        <color rgb="00BBC9D3"/>
       </bottom>
     </border>
     <border>
@@ -122,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -135,16 +140,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -156,24 +158,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -646,7 +648,13 @@
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="9" t="n"/>
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -667,32 +675,32 @@
           <t>Type de mandat (cocher)</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>SAJ</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>SPJ</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr">
+      <c r="G14" s="10" t="inlineStr">
         <is>
           <t>Tribunal</t>
         </is>
@@ -732,32 +740,32 @@
           <t>Prise en charge (cocher)</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>F.A.</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Frais</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>SAAF</t>
         </is>
@@ -769,32 +777,32 @@
           <t>Allocation forfaitaire allouée à (cocher)</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Maman</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Papa</t>
         </is>
       </c>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Enfant</t>
         </is>
@@ -808,7 +816,13 @@
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
-      <c r="A20" s="9" t="n"/>
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -824,127 +838,119 @@
       <c r="G23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Besoin</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="13" t="inlineStr">
         <is>
           <t>Objectifs de travail (court / moyen / long terme)</t>
         </is>
       </c>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="13" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
     </row>
     <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Besoins physiologiques – sommeil – alimentation – santé (suivi médical, vaccins, dentiste…)</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="9" t="n"/>
+      <c r="C25" s="6" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="9" t="n"/>
+      <c r="E25" s="6" t="n"/>
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="7" t="n"/>
     </row>
     <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Sécurité – protection – stabilité (repères, limites)</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="9" t="n"/>
+      <c r="C26" s="6" t="n"/>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="9" t="n"/>
+      <c r="E26" s="6" t="n"/>
       <c r="F26" s="7" t="n"/>
       <c r="G26" s="7" t="n"/>
     </row>
     <row r="27" ht="46" customHeight="1">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>Affectif – relation d'attachement – appartenance</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="9" t="n"/>
+      <c r="C27" s="6" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="9" t="n"/>
+      <c r="E27" s="6" t="n"/>
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="7" t="n"/>
     </row>
     <row r="28" ht="46" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Estime de soi – épanouissement</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="9" t="n"/>
+      <c r="C28" s="6" t="n"/>
       <c r="D28" s="7" t="n"/>
-      <c r="E28" s="9" t="n"/>
+      <c r="E28" s="6" t="n"/>
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="7" t="n"/>
     </row>
     <row r="29" ht="46" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>Apprentissage – formation</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="9" t="n"/>
+      <c r="C29" s="6" t="n"/>
       <c r="D29" s="7" t="n"/>
-      <c r="E29" s="9" t="n"/>
+      <c r="E29" s="6" t="n"/>
       <c r="F29" s="7" t="n"/>
       <c r="G29" s="7" t="n"/>
     </row>
     <row r="30" ht="46" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>Développement des compétences</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="9" t="n"/>
+      <c r="C30" s="6" t="n"/>
       <c r="D30" s="7" t="n"/>
-      <c r="E30" s="9" t="n"/>
+      <c r="E30" s="6" t="n"/>
       <c r="F30" s="7" t="n"/>
       <c r="G30" s="7" t="n"/>
     </row>
     <row r="31" ht="46" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>Appartenance à un réseau social</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="9" t="n"/>
+      <c r="C31" s="6" t="n"/>
       <c r="D31" s="7" t="n"/>
-      <c r="E31" s="9" t="n"/>
+      <c r="E31" s="6" t="n"/>
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="7" t="n"/>
     </row>
     <row r="32" ht="46" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>Développer son autonomie – sa responsabilité</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="9" t="n"/>
+      <c r="C32" s="6" t="n"/>
       <c r="D32" s="7" t="n"/>
-      <c r="E32" s="9" t="n"/>
+      <c r="E32" s="6" t="n"/>
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="7" t="n"/>
     </row>
@@ -962,166 +968,155 @@
       <c r="G35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>Élément</t>
         </is>
       </c>
-      <c r="B36" s="13" t="n"/>
-      <c r="C36" s="12" t="inlineStr">
+      <c r="B36" s="12" t="n"/>
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="D36" s="13" t="n"/>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="D36" s="12" t="n"/>
+      <c r="E36" s="13" t="inlineStr">
         <is>
           <t>Objectifs de travail (court / moyen / long terme)</t>
         </is>
       </c>
-      <c r="F36" s="13" t="n"/>
-      <c r="G36" s="13" t="n"/>
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="12" t="n"/>
     </row>
     <row r="37" ht="46" customHeight="1">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>Situation actuelle</t>
         </is>
       </c>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="9" t="n"/>
+      <c r="C37" s="6" t="n"/>
       <c r="D37" s="7" t="n"/>
-      <c r="E37" s="9" t="n"/>
+      <c r="E37" s="6" t="n"/>
       <c r="F37" s="7" t="n"/>
       <c r="G37" s="7" t="n"/>
     </row>
     <row r="38" ht="46" customHeight="1">
-      <c r="A38" s="15" t="inlineStr">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>Disponibilité</t>
         </is>
       </c>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="9" t="n"/>
+      <c r="C38" s="6" t="n"/>
       <c r="D38" s="7" t="n"/>
-      <c r="E38" s="9" t="n"/>
+      <c r="E38" s="6" t="n"/>
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="7" t="n"/>
     </row>
     <row r="39" ht="46" customHeight="1">
-      <c r="A39" s="15" t="inlineStr">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>Collaboration</t>
         </is>
       </c>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="9" t="n"/>
+      <c r="C39" s="6" t="n"/>
       <c r="D39" s="7" t="n"/>
-      <c r="E39" s="9" t="n"/>
+      <c r="E39" s="6" t="n"/>
       <c r="F39" s="7" t="n"/>
       <c r="G39" s="7" t="n"/>
     </row>
     <row r="40" ht="46" customHeight="1">
-      <c r="A40" s="15" t="inlineStr">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>Ouverture à la F.O.</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="9" t="n"/>
+      <c r="C40" s="6" t="n"/>
       <c r="D40" s="7" t="n"/>
-      <c r="E40" s="9" t="n"/>
+      <c r="E40" s="6" t="n"/>
       <c r="F40" s="7" t="n"/>
       <c r="G40" s="7" t="n"/>
     </row>
     <row r="41" ht="46" customHeight="1">
-      <c r="A41" s="15" t="inlineStr">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>À l'extérieur</t>
         </is>
       </c>
-      <c r="B41" s="7" t="n"/>
-      <c r="C41" s="9" t="n"/>
+      <c r="C41" s="6" t="n"/>
       <c r="D41" s="7" t="n"/>
-      <c r="E41" s="9" t="n"/>
+      <c r="E41" s="6" t="n"/>
       <c r="F41" s="7" t="n"/>
       <c r="G41" s="7" t="n"/>
     </row>
     <row r="42" ht="46" customHeight="1">
-      <c r="A42" s="15" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>Éducation (souple, rigide…)</t>
         </is>
       </c>
-      <c r="B42" s="7" t="n"/>
-      <c r="C42" s="9" t="n"/>
+      <c r="C42" s="6" t="n"/>
       <c r="D42" s="7" t="n"/>
-      <c r="E42" s="9" t="n"/>
+      <c r="E42" s="6" t="n"/>
       <c r="F42" s="7" t="n"/>
       <c r="G42" s="7" t="n"/>
     </row>
     <row r="43" ht="46" customHeight="1">
-      <c r="A43" s="15" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>Remise en question</t>
         </is>
       </c>
-      <c r="B43" s="7" t="n"/>
-      <c r="C43" s="9" t="n"/>
+      <c r="C43" s="6" t="n"/>
       <c r="D43" s="7" t="n"/>
-      <c r="E43" s="9" t="n"/>
+      <c r="E43" s="6" t="n"/>
       <c r="F43" s="7" t="n"/>
       <c r="G43" s="7" t="n"/>
     </row>
     <row r="44" ht="46" customHeight="1">
-      <c r="A44" s="15" t="inlineStr">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>Relations famille élargie (fratrie, grands-parents…)</t>
         </is>
       </c>
-      <c r="B44" s="7" t="n"/>
-      <c r="C44" s="9" t="n"/>
+      <c r="C44" s="6" t="n"/>
       <c r="D44" s="7" t="n"/>
-      <c r="E44" s="9" t="n"/>
+      <c r="E44" s="6" t="n"/>
       <c r="F44" s="7" t="n"/>
       <c r="G44" s="7" t="n"/>
     </row>
     <row r="45" ht="46" customHeight="1">
-      <c r="A45" s="15" t="inlineStr">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>Réseau</t>
         </is>
       </c>
-      <c r="B45" s="7" t="n"/>
-      <c r="C45" s="9" t="n"/>
+      <c r="C45" s="6" t="n"/>
       <c r="D45" s="7" t="n"/>
-      <c r="E45" s="9" t="n"/>
+      <c r="E45" s="6" t="n"/>
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="7" t="n"/>
     </row>
     <row r="46" ht="46" customHeight="1">
-      <c r="A46" s="15" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Couple</t>
         </is>
       </c>
-      <c r="B46" s="7" t="n"/>
-      <c r="C46" s="9" t="n"/>
+      <c r="C46" s="6" t="n"/>
       <c r="D46" s="7" t="n"/>
-      <c r="E46" s="9" t="n"/>
+      <c r="E46" s="6" t="n"/>
       <c r="F46" s="7" t="n"/>
       <c r="G46" s="7" t="n"/>
     </row>
     <row r="47" ht="46" customHeight="1">
-      <c r="A47" s="15" t="inlineStr">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>Rôles parentaux</t>
         </is>
       </c>
-      <c r="B47" s="7" t="n"/>
-      <c r="C47" s="9" t="n"/>
+      <c r="C47" s="6" t="n"/>
       <c r="D47" s="7" t="n"/>
-      <c r="E47" s="9" t="n"/>
+      <c r="E47" s="6" t="n"/>
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="7" t="n"/>
     </row>
@@ -1139,101 +1134,95 @@
       <c r="G50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="12" t="inlineStr">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Élément</t>
         </is>
       </c>
-      <c r="B51" s="13" t="n"/>
-      <c r="C51" s="12" t="inlineStr">
+      <c r="B51" s="12" t="n"/>
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="D51" s="13" t="n"/>
-      <c r="E51" s="14" t="inlineStr">
+      <c r="D51" s="12" t="n"/>
+      <c r="E51" s="13" t="inlineStr">
         <is>
           <t>Objectifs de travail (court / moyen / long terme)</t>
         </is>
       </c>
-      <c r="F51" s="13" t="n"/>
-      <c r="G51" s="13" t="n"/>
+      <c r="F51" s="12" t="n"/>
+      <c r="G51" s="12" t="n"/>
     </row>
     <row r="52" ht="46" customHeight="1">
-      <c r="A52" s="15" t="inlineStr">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>Situation actuelle</t>
         </is>
       </c>
-      <c r="B52" s="7" t="n"/>
-      <c r="C52" s="9" t="n"/>
+      <c r="C52" s="6" t="n"/>
       <c r="D52" s="7" t="n"/>
-      <c r="E52" s="9" t="n"/>
+      <c r="E52" s="6" t="n"/>
       <c r="F52" s="7" t="n"/>
       <c r="G52" s="7" t="n"/>
     </row>
     <row r="53" ht="46" customHeight="1">
-      <c r="A53" s="15" t="inlineStr">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>Perception des parents</t>
         </is>
       </c>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="9" t="n"/>
+      <c r="C53" s="6" t="n"/>
       <c r="D53" s="7" t="n"/>
-      <c r="E53" s="9" t="n"/>
+      <c r="E53" s="6" t="n"/>
       <c r="F53" s="7" t="n"/>
       <c r="G53" s="7" t="n"/>
     </row>
     <row r="54" ht="46" customHeight="1">
-      <c r="A54" s="15" t="inlineStr">
+      <c r="A54" s="14" t="inlineStr">
         <is>
           <t>Collaboration</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="9" t="n"/>
+      <c r="C54" s="6" t="n"/>
       <c r="D54" s="7" t="n"/>
-      <c r="E54" s="9" t="n"/>
+      <c r="E54" s="6" t="n"/>
       <c r="F54" s="7" t="n"/>
       <c r="G54" s="7" t="n"/>
     </row>
     <row r="55" ht="46" customHeight="1">
-      <c r="A55" s="15" t="inlineStr">
+      <c r="A55" s="14" t="inlineStr">
         <is>
           <t>Remise en question</t>
         </is>
       </c>
-      <c r="B55" s="7" t="n"/>
-      <c r="C55" s="9" t="n"/>
+      <c r="C55" s="6" t="n"/>
       <c r="D55" s="7" t="n"/>
-      <c r="E55" s="9" t="n"/>
+      <c r="E55" s="6" t="n"/>
       <c r="F55" s="7" t="n"/>
       <c r="G55" s="7" t="n"/>
     </row>
     <row r="56" ht="46" customHeight="1">
-      <c r="A56" s="15" t="inlineStr">
+      <c r="A56" s="14" t="inlineStr">
         <is>
           <t>D.R.P.</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n"/>
-      <c r="C56" s="9" t="n"/>
+      <c r="C56" s="6" t="n"/>
       <c r="D56" s="7" t="n"/>
-      <c r="E56" s="9" t="n"/>
+      <c r="E56" s="6" t="n"/>
       <c r="F56" s="7" t="n"/>
       <c r="G56" s="7" t="n"/>
     </row>
     <row r="57" ht="46" customHeight="1">
-      <c r="A57" s="15" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>Autre</t>
         </is>
       </c>
-      <c r="B57" s="7" t="n"/>
-      <c r="C57" s="9" t="n"/>
+      <c r="C57" s="6" t="n"/>
       <c r="D57" s="7" t="n"/>
-      <c r="E57" s="9" t="n"/>
+      <c r="E57" s="6" t="n"/>
       <c r="F57" s="7" t="n"/>
       <c r="G57" s="7" t="n"/>
     </row>
@@ -1251,28 +1240,28 @@
       <c r="G60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="12" t="inlineStr">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B61" s="13" t="n"/>
-      <c r="C61" s="13" t="n"/>
-      <c r="D61" s="13" t="n"/>
-      <c r="E61" s="14" t="inlineStr">
+      <c r="B61" s="12" t="n"/>
+      <c r="C61" s="12" t="n"/>
+      <c r="D61" s="12" t="n"/>
+      <c r="E61" s="13" t="inlineStr">
         <is>
           <t>Objectifs de travail (court / moyen / long terme)</t>
         </is>
       </c>
-      <c r="F61" s="13" t="n"/>
-      <c r="G61" s="13" t="n"/>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="12" t="n"/>
     </row>
     <row r="62" ht="56" customHeight="1">
-      <c r="A62" s="9" t="n"/>
+      <c r="A62" s="6" t="n"/>
       <c r="B62" s="7" t="n"/>
       <c r="C62" s="7" t="n"/>
       <c r="D62" s="7" t="n"/>
-      <c r="E62" s="9" t="n"/>
+      <c r="E62" s="6" t="n"/>
       <c r="F62" s="7" t="n"/>
       <c r="G62" s="7" t="n"/>
     </row>
@@ -1295,7 +1284,7 @@
           <t>Enfant</t>
         </is>
       </c>
-      <c r="C66" s="9" t="n"/>
+      <c r="C66" s="6" t="n"/>
       <c r="D66" s="7" t="n"/>
       <c r="E66" s="7" t="n"/>
       <c r="F66" s="7" t="n"/>
@@ -1307,7 +1296,7 @@
           <t>Famille d'accueil</t>
         </is>
       </c>
-      <c r="C67" s="9" t="n"/>
+      <c r="C67" s="6" t="n"/>
       <c r="D67" s="7" t="n"/>
       <c r="E67" s="7" t="n"/>
       <c r="F67" s="7" t="n"/>
@@ -1319,7 +1308,7 @@
           <t>Famille d'origine</t>
         </is>
       </c>
-      <c r="C68" s="9" t="n"/>
+      <c r="C68" s="6" t="n"/>
       <c r="D68" s="7" t="n"/>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="7" t="n"/>
@@ -1331,7 +1320,7 @@
           <t>D.R.P.</t>
         </is>
       </c>
-      <c r="C69" s="9" t="n"/>
+      <c r="C69" s="6" t="n"/>
       <c r="D69" s="7" t="n"/>
       <c r="E69" s="7" t="n"/>
       <c r="F69" s="7" t="n"/>
@@ -1343,7 +1332,7 @@
           <t>Mandat</t>
         </is>
       </c>
-      <c r="C70" s="9" t="n"/>
+      <c r="C70" s="6" t="n"/>
       <c r="D70" s="7" t="n"/>
       <c r="E70" s="7" t="n"/>
       <c r="F70" s="7" t="n"/>
@@ -1363,39 +1352,39 @@
       <c r="G73" s="4" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="16" t="inlineStr">
+      <c r="A74" s="15" t="inlineStr">
         <is>
           <t>Enfants</t>
         </is>
       </c>
-      <c r="B74" s="16" t="inlineStr">
+      <c r="B74" s="15" t="inlineStr">
         <is>
           <t>Pts</t>
         </is>
       </c>
-      <c r="C74" s="16" t="inlineStr">
+      <c r="C74" s="15" t="inlineStr">
         <is>
           <t>F.A.</t>
         </is>
       </c>
-      <c r="D74" s="16" t="inlineStr">
+      <c r="D74" s="15" t="inlineStr">
         <is>
           <t>Pts</t>
         </is>
       </c>
-      <c r="E74" s="16" t="inlineStr">
+      <c r="E74" s="15" t="inlineStr">
         <is>
           <t>F.O.</t>
         </is>
       </c>
-      <c r="F74" s="16" t="inlineStr">
+      <c r="F74" s="15" t="inlineStr">
         <is>
           <t>Pts</t>
         </is>
       </c>
     </row>
     <row r="75" ht="78" customHeight="1">
-      <c r="A75" s="17" t="inlineStr">
+      <c r="A75" s="16" t="inlineStr">
         <is>
           <t>D.R.P.
   • Nombre
@@ -1405,22 +1394,22 @@
   • Type</t>
         </is>
       </c>
-      <c r="B75" s="18" t="n"/>
-      <c r="C75" s="17" t="inlineStr">
+      <c r="B75" s="17" t="n"/>
+      <c r="C75" s="16" t="inlineStr">
         <is>
           <t>D.R.P.</t>
         </is>
       </c>
-      <c r="D75" s="18" t="n"/>
-      <c r="E75" s="17" t="inlineStr">
+      <c r="D75" s="17" t="n"/>
+      <c r="E75" s="16" t="inlineStr">
         <is>
           <t>D.R.P.</t>
         </is>
       </c>
-      <c r="F75" s="18" t="n"/>
+      <c r="F75" s="17" t="n"/>
     </row>
     <row r="76" ht="70" customHeight="1">
-      <c r="A76" s="17" t="inlineStr">
+      <c r="A76" s="16" t="inlineStr">
         <is>
           <t>État de l'enfant :
   • Scolaire
@@ -1429,109 +1418,109 @@
   • Développement</t>
         </is>
       </c>
-      <c r="B76" s="18" t="n"/>
-      <c r="C76" s="17" t="inlineStr">
+      <c r="B76" s="17" t="n"/>
+      <c r="C76" s="16" t="inlineStr">
         <is>
           <t>Administratif
 Financier</t>
         </is>
       </c>
-      <c r="D76" s="18" t="n"/>
-      <c r="E76" s="17" t="inlineStr">
+      <c r="D76" s="17" t="n"/>
+      <c r="E76" s="16" t="inlineStr">
         <is>
           <t>Retour des parents</t>
         </is>
       </c>
-      <c r="F76" s="18" t="n"/>
+      <c r="F76" s="17" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="17" t="inlineStr">
+      <c r="A77" s="16" t="inlineStr">
         <is>
           <t>Bilan 6 mois</t>
         </is>
       </c>
-      <c r="B77" s="18" t="n"/>
-      <c r="C77" s="17" t="inlineStr">
+      <c r="B77" s="17" t="n"/>
+      <c r="C77" s="16" t="inlineStr">
         <is>
           <t>Bilan 6 mois</t>
         </is>
       </c>
-      <c r="D77" s="18" t="n"/>
-      <c r="E77" s="17" t="inlineStr">
+      <c r="D77" s="17" t="n"/>
+      <c r="E77" s="16" t="inlineStr">
         <is>
           <t>Bilan 6 mois</t>
         </is>
       </c>
-      <c r="F77" s="18" t="n"/>
+      <c r="F77" s="17" t="n"/>
     </row>
     <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="17" t="inlineStr">
+      <c r="A78" s="16" t="inlineStr">
         <is>
           <t>Réintégration</t>
         </is>
       </c>
-      <c r="B78" s="18" t="n"/>
-      <c r="C78" s="17" t="inlineStr">
+      <c r="B78" s="17" t="n"/>
+      <c r="C78" s="16" t="inlineStr">
         <is>
           <t>Réintégration</t>
         </is>
       </c>
-      <c r="D78" s="18" t="n"/>
-      <c r="E78" s="17" t="inlineStr">
+      <c r="D78" s="17" t="n"/>
+      <c r="E78" s="16" t="inlineStr">
         <is>
           <t>Réintégration</t>
         </is>
       </c>
-      <c r="F78" s="18" t="n"/>
+      <c r="F78" s="17" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="17" t="inlineStr">
+      <c r="A79" s="16" t="inlineStr">
         <is>
           <t>Préparation à la majorité</t>
         </is>
       </c>
-      <c r="B79" s="18" t="n"/>
-      <c r="C79" s="17" t="inlineStr">
+      <c r="B79" s="17" t="n"/>
+      <c r="C79" s="16" t="inlineStr">
         <is>
           <t>Préparation à la majorité</t>
         </is>
       </c>
-      <c r="D79" s="18" t="n"/>
-      <c r="E79" s="17" t="inlineStr">
+      <c r="D79" s="17" t="n"/>
+      <c r="E79" s="16" t="inlineStr">
         <is>
           <t>Préparation à la majorité</t>
         </is>
       </c>
-      <c r="F79" s="18" t="n"/>
+      <c r="F79" s="17" t="n"/>
     </row>
     <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="17" t="inlineStr">
+      <c r="A80" s="16" t="inlineStr">
         <is>
           <t>Travail de l'histoire</t>
         </is>
       </c>
-      <c r="B80" s="18" t="n"/>
-      <c r="C80" s="17" t="inlineStr">
+      <c r="B80" s="17" t="n"/>
+      <c r="C80" s="16" t="inlineStr">
         <is>
           <t>Recherche activités</t>
         </is>
       </c>
-      <c r="D80" s="18" t="n"/>
-      <c r="E80" s="17" t="inlineStr">
+      <c r="D80" s="17" t="n"/>
+      <c r="E80" s="16" t="inlineStr">
         <is>
           <t>Écrits autorité</t>
         </is>
       </c>
-      <c r="F80" s="18" t="n"/>
+      <c r="F80" s="17" t="n"/>
     </row>
     <row r="81" ht="60" customHeight="1">
-      <c r="A81" s="17" t="inlineStr">
+      <c r="A81" s="16" t="inlineStr">
         <is>
           <t>Autorité (écrits)</t>
         </is>
       </c>
-      <c r="B81" s="18" t="n"/>
-      <c r="C81" s="17" t="inlineStr">
+      <c r="B81" s="17" t="n"/>
+      <c r="C81" s="16" t="inlineStr">
         <is>
           <t>Besoin de sécurité
   • Accompagnement
@@ -1539,45 +1528,45 @@
   • Autorité</t>
         </is>
       </c>
-      <c r="D81" s="18" t="n"/>
-      <c r="E81" s="17" t="inlineStr"/>
-      <c r="F81" s="18" t="n"/>
+      <c r="D81" s="17" t="n"/>
+      <c r="E81" s="16" t="inlineStr"/>
+      <c r="F81" s="17" t="n"/>
     </row>
     <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="17" t="inlineStr">
+      <c r="A82" s="16" t="inlineStr">
         <is>
           <t>Déplacements</t>
         </is>
       </c>
-      <c r="B82" s="18" t="n"/>
-      <c r="C82" s="17" t="inlineStr"/>
-      <c r="D82" s="18" t="n"/>
-      <c r="E82" s="17" t="inlineStr"/>
-      <c r="F82" s="18" t="n"/>
+      <c r="B82" s="17" t="n"/>
+      <c r="C82" s="16" t="inlineStr"/>
+      <c r="D82" s="17" t="n"/>
+      <c r="E82" s="16" t="inlineStr"/>
+      <c r="F82" s="17" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="19" t="inlineStr">
+      <c r="A83" s="18" t="inlineStr">
         <is>
           <t>TOTAUX</t>
         </is>
       </c>
-      <c r="B83" s="20">
+      <c r="B83" s="19">
         <f>SUM(B75:B82)</f>
         <v/>
       </c>
-      <c r="C83" s="21" t="n"/>
-      <c r="D83" s="20">
+      <c r="C83" s="20" t="n"/>
+      <c r="D83" s="19">
         <f>SUM(D75:D82)</f>
         <v/>
       </c>
-      <c r="E83" s="21" t="n"/>
-      <c r="F83" s="20">
+      <c r="E83" s="20" t="n"/>
+      <c r="F83" s="19">
         <f>SUM(F75:F82)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CDB4"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CDB4"/>
   <mergeCells count="85">
     <mergeCell ref="C68:G68"/>
     <mergeCell ref="F16:G16"/>

</xml_diff>